<commit_message>
worked on some more problems, renamed marsh-data.py to analysis.py
</commit_message>
<xml_diff>
--- a/GaltonFamilies-1886.xlsx
+++ b/GaltonFamilies-1886.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10412"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Keys/Projects/prob-and-stat-project-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A6BF90-ED92-0145-8715-83149F972627}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A10E810D-BE9D-B54B-BB41-DEEFF349186F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="15800" windowHeight="10840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5160" yWindow="2760" windowWidth="15800" windowHeight="10840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GaltonFamilies" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 

</xml_diff>